<commit_message>
feat: v1.1 — history view + free-text surface
Backend:
- blocker_text, manager_needs, risks_text pass through to JSON output
- strip() moved into Pydantic field_validator on Raw* models
- synthetic generator uses varied sample texts per field
- 95 tests (+11), incl. whitespace-only edge case

Frontend:
- History view (3rd toggle): team health bar + RAG strip + sparklines
  per consultant across all archived weekly/monthly periods
- SituationBlock: blocker_text + risks_text quoted inline in action items
- ConsultantCards: manager_needs + risks_text in expanded monthly rows
- 8 weekly + 6 monthly synthetic periods for history testing

Docs: CLAUDE.md updated — component tree, layout, History view section
</commit_message>
<xml_diff>
--- a/backend/data/synthetic/pulse_data.xlsx
+++ b/backend/data/synthetic/pulse_data.xlsx
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -479,7 +479,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -505,7 +505,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -514,24 +514,28 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Waiting for safety approval from functional safety team.</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -540,7 +544,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -557,7 +561,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -566,28 +570,24 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Toolchain access issue</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -613,7 +613,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -632,14 +632,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -648,18 +648,14 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Toolchain access issue</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>No</t>
@@ -669,7 +665,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -695,7 +691,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -704,14 +700,18 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Customer portal credentials expired — request pending 4 days.</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>No</t>
@@ -721,7 +721,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -730,14 +730,18 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Waiting for safety approval from functional safety team.</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>No</t>
@@ -747,7 +751,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -756,7 +760,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -773,7 +777,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -782,24 +786,28 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Waiting for safety approval from functional safety team.</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -808,14 +816,18 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Customer portal credentials expired — request pending 4 days.</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>No</t>
@@ -825,7 +837,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -834,7 +846,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -851,7 +863,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -877,7 +889,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -886,7 +898,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -964,7 +976,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -973,29 +985,29 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1004,29 +1016,33 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
         <v>5</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Escalation on tooling blockers takes too long.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1035,29 +1051,33 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Would like a 1:1 to discuss next project rotation.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1066,29 +1086,33 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Would like a 1:1 to discuss next project rotation.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1103,23 +1127,23 @@
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
         <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1128,29 +1152,33 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>4</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Escalation on tooling blockers takes too long.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1159,29 +1187,29 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1190,16 +1218,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
         <v>1</v>
@@ -1207,12 +1235,16 @@
       <c r="H9" t="n">
         <v>5</v>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Need clarity on Q3 scope — feature list keeps changing.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1221,29 +1253,33 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
         <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Escalation on tooling blockers takes too long.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1252,10 +1288,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
@@ -1267,14 +1303,18 @@
         <v>4</v>
       </c>
       <c r="H11" t="n">
-        <v>5</v>
-      </c>
-      <c r="I11" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Need clarity on Q3 scope — feature list keeps changing.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1283,29 +1323,33 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>5</v>
-      </c>
-      <c r="I12" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Would like a 1:1 to discuss next project rotation.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1314,29 +1358,33 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H13" t="n">
-        <v>5</v>
-      </c>
-      <c r="I13" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Would like a 1:1 to discuss next project rotation.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1345,29 +1393,33 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Training budget for ISO 26262 refresher would help.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1379,26 +1431,30 @@
         <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
         <v>3</v>
       </c>
       <c r="H15" t="n">
-        <v>4</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Need clarity on Q3 scope — feature list keeps changing.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1407,29 +1463,33 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
-      <c r="I16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Need clarity on Q3 scope — feature list keeps changing.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1438,29 +1498,33 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
         <v>5</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H17" t="n">
-        <v>4</v>
-      </c>
-      <c r="I17" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Need clarity on Q3 scope — feature list keeps changing.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1469,16 +1533,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n">
         <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
@@ -1486,7 +1550,11 @@
       <c r="H18" t="n">
         <v>2</v>
       </c>
-      <c r="I18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Would like a 1:1 to discuss next project rotation.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1542,7 +1610,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1554,20 +1622,24 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
         <v>3</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Customer escalated twice last week — needs executive attention.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1576,23 +1648,23 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1601,7 +1673,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
         <v>3</v>
@@ -1612,12 +1684,16 @@
       <c r="F4" t="n">
         <v>5</v>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Technical debt blocking feature delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1626,23 +1702,27 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Deadline at risk due to supplier delay on module X.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1651,10 +1731,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -1662,12 +1742,16 @@
       <c r="F6" t="n">
         <v>4</v>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Technical debt blocking feature delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1676,23 +1760,23 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1704,20 +1788,20 @@
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1726,13 +1810,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
         <v>3</v>
@@ -1742,7 +1826,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1751,23 +1835,27 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>3</v>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Customer escalated twice last week — needs executive attention.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1782,17 +1870,21 @@
         <v>5</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Technical debt blocking feature delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1801,23 +1893,27 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Consultant overloaded on two parallel projects.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1826,23 +1922,23 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1857,17 +1953,17 @@
         <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1876,23 +1972,27 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Customer escalated twice last week — needs executive attention.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1904,20 +2004,24 @@
         <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
         <v>5</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Customer escalated twice last week — needs executive attention.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1926,23 +2030,27 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
         <v>5</v>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Technical debt blocking feature delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>14/04/2026 10:00</t>
+          <t>15/11/2025 10:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1951,18 +2059,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Technical debt blocking feature delivery.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>